<commit_message>
Update: Google Ads Report Editor 5-Row and 5-Metric Tree Table Layout
</commit_message>
<xml_diff>
--- a/NMC_Hospital_Master_Template.xlsx
+++ b/NMC_Hospital_Master_Template.xlsx
@@ -446,33 +446,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="54" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="43" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
     <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="27" customWidth="1" min="22" max="22"/>
-    <col width="25" customWidth="1" min="23" max="23"/>
-    <col width="15" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,95 +495,55 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Match type</t>
+          <t>Impressions</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Quality score</t>
+          <t>Clicks</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Exp. CTR</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Ad relevance</t>
+          <t>Conversions</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Landing page exp.</t>
+          <t>Avg. CPC</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Impressions</t>
+          <t>CTR</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Clicks</t>
+          <t>Cost / conv.</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>CTR</t>
+          <t>Conv. rate</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Avg. CPC</t>
+          <t>Search impr. share</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Search lost IS (rank)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Conversions</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Cost / conv.</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Conv. rate</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Search impr. share</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Search top IS</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Search abs. top IS</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Search lost IS (budget)</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Search lost IS (rank)</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Phone calls</t>
         </is>
@@ -615,7 +567,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Internal Medicine - Exact</t>
+          <t>Internal Medicine - Samnan High Intent</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -623,83 +575,45 @@
           <t>internal medicine doctor samnan sharjah</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Exact</t>
-        </is>
+      <c r="F2" t="n">
+        <v>310</v>
       </c>
       <c r="G2" t="n">
-        <v>9</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>310</v>
+        <v>32</v>
+      </c>
+      <c r="H2" t="n">
+        <v>268.8</v>
+      </c>
+      <c r="I2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J2" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>10.32%</t>
+        </is>
       </c>
       <c r="L2" t="n">
-        <v>32</v>
+        <v>44.8</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>10.32%</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="O2" t="n">
-        <v>268.8</v>
+          <t>18.75%</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>88.0%</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
       </c>
       <c r="P2" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>18.75%</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>88.0%</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>88.0%</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>62.0%</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>8.0%</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>4.0%</t>
-        </is>
-      </c>
-      <c r="X2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -729,83 +643,45 @@
           <t>best cardiologist in abu dhabi</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Exact</t>
-        </is>
+      <c r="F3" t="n">
+        <v>320</v>
       </c>
       <c r="G3" t="n">
-        <v>9</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>320</v>
+        <v>30</v>
+      </c>
+      <c r="H3" t="n">
+        <v>426</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>9.38%</t>
+        </is>
       </c>
       <c r="L3" t="n">
-        <v>30</v>
+        <v>85.2</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>9.38%</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="O3" t="n">
-        <v>426</v>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>84.0%</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>5.5%</t>
+        </is>
       </c>
       <c r="P3" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>16.67%</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>84.0%</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>82.5%</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>54.0%</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>12.0%</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>5.5%</t>
-        </is>
-      </c>
-      <c r="X3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -835,83 +711,45 @@
           <t>knee replacement surgeon dubai</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Exact</t>
-        </is>
+      <c r="F4" t="n">
+        <v>280</v>
       </c>
       <c r="G4" t="n">
-        <v>9</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>280</v>
+        <v>26</v>
+      </c>
+      <c r="H4" t="n">
+        <v>582.4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>9.28%</t>
+        </is>
       </c>
       <c r="L4" t="n">
-        <v>26</v>
+        <v>116.48</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>9.28%</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="O4" t="n">
-        <v>582.4</v>
+          <t>19.23%</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>86.0%</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>5.0%</t>
+        </is>
       </c>
       <c r="P4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>116.48</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>19.23%</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>86.0%</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>85.0%</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>59.0%</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>9.0%</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>5.0%</t>
-        </is>
-      </c>
-      <c r="X4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -941,83 +779,45 @@
           <t>cardiologist in sharjah royal hospital</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Exact</t>
-        </is>
+      <c r="F5" t="n">
+        <v>290</v>
       </c>
       <c r="G5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>290</v>
+        <v>28</v>
+      </c>
+      <c r="H5" t="n">
+        <v>358.4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>9.66%</t>
+        </is>
       </c>
       <c r="L5" t="n">
-        <v>28</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>9.66%</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="O5" t="n">
-        <v>358.4</v>
+          <t>17.86%</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>87.0%</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>6.0%</t>
+        </is>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>71.68000000000001</v>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>17.86%</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>87.0%</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>87.0%</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>61.0%</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>7.0%</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>6.0%</t>
-        </is>
-      </c>
-      <c r="X5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1047,83 +847,45 @@
           <t>pediatrician buhaira corniche sharjah</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Exact</t>
-        </is>
+      <c r="F6" t="n">
+        <v>360</v>
       </c>
       <c r="G6" t="n">
-        <v>9</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Above average</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>360</v>
+        <v>38</v>
+      </c>
+      <c r="H6" t="n">
+        <v>285</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>10.56%</t>
+        </is>
       </c>
       <c r="L6" t="n">
-        <v>38</v>
+        <v>35.62</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>10.56%</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="O6" t="n">
-        <v>285</v>
+          <t>21.05%</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>90.0%</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>5.0%</t>
+        </is>
       </c>
       <c r="P6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>35.62</v>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>21.05%</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>90.0%</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>90.0%</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>69.0%</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>5.0%</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>5.0%</t>
-        </is>
-      </c>
-      <c r="X6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1592,17 +1354,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="53" customWidth="1" min="1" max="1"/>
-    <col width="273" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="1" max="1"/>
+    <col width="118" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Google Ads Report Editor Tree Table Configuration</t>
+          <t>Google Ads Report Editor Tree Table Configuration (5 Rows + 5 Metrics)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -1614,24 +1376,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Row Hierarchy (First 4 Dimensions):</t>
+          <t>Row Dimensions in Google Ads Tree Table (Drag these 5 to Rows):</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1. Day  |  2. Campaign  |  3. Account  |  4. Ad group</t>
+          <t>1. Day (Date)  |  2. Campaign  |  3. Account  |  4. Ad group  |  5. Search keyword</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Metric Columns:</t>
+          <t>Metric Columns in Google Ads Tree Table (Drag these 5 to Columns):</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Search keyword, Match type, Quality score, Exp. CTR, Ad relevance, Landing page exp., Impr., Clicks, CTR, Avg. CPC, Cost, Conv., Cost / conv., Conv. rate, Search impr. share, Search top IS, Search abs. top IS, Search lost IS (budget), Search lost IS (rank), Phone calls</t>
+          <t>1. Impressions  |  2. Clicks  |  3. Cost (AED)  |  4. Conversions  |  5. Avg. CPC</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1404,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dashboard Connection:</t>
+          <t>Automated Derived Metrics Calculated by Dashboard:</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Directly paste rows into Google_Ads_Data tab and click '🚀 NMC Sync &gt; 🔄 Sync Data to Dashboard'.</t>
+          <t>CTR %, Cost Per Conv (CPA), Conv. Rate %, Confirmed Bookings, CPBA, Show-Up Rate %, Speciality &amp; Branch Extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Capacity:</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pre-configured for Lakhs of rows (100,000 - 500,000+ rows) across both tabs.</t>
         </is>
       </c>
     </row>

</xml_diff>